<commit_message>
Fix negative/01 validation for CORE-000579
The engine bug (empty-dataset insert raising an exception) was already
fixed upstream in cdisc-rules-engine and is included in the pinned
submodule commit, so the checked-in results.json was just a stale
fixture from before that fix. Regenerated it, and added the missing
Validation-sheet row so the dataset-level "Dataset has no record."
error is fully validated.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/rules/CORE-000579/negative/01/data/unit-test-coreid-CG0408-negative.xlsx
+++ b/rules/CORE-000579/negative/01/data/unit-test-coreid-CG0408-negative.xlsx
@@ -529,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -561,6 +561,36 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ae.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>records_in_dataset</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1052,6 @@
       <c r="T5" s="4" t="n"/>
       <c r="U5" s="4" t="n"/>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="T7" s="4" t="n"/>
     </row>

</xml_diff>